<commit_message>
Add Stroke Index to Rounds, Tee Colour to Courses, verified Pupuke data
Rounds tab (now 24 cols):
- Stroke Index added as col 7 (between Distance and Score)

Courses tab (now 7 cols):
- Tee Colour added as col 3 -- par/distance vary per tee
- Pupuke White tee stroke indexes corrected

README fully updated with numbered column guides, verified Pupuke
table, and updated status section.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:X5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -456,23 +456,24 @@
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="11" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="11" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
     <col width="13" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="60" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="12" customWidth="1" min="23" max="23"/>
+    <col width="60" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -508,89 +509,94 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Stroke Index</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Strokes</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Putts</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Penalties</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Tee Club</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pick Up</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Sentiment</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Woods</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Hybrids</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Long Irons
 (5-7)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Short Irons
 (8-P)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Wedges
 (GW/SW/LW)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Putter</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Playing
 Handicap</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Tee Colour</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -619,65 +625,66 @@
       <c r="F2" s="3" t="n">
         <v>5188</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>85</v>
-      </c>
+      <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n">
         <v>85</v>
       </c>
       <c r="I2" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="J2" s="3" t="n">
         <v>32</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K2" s="3" t="inlineStr"/>
       <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="O2" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr"/>
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="R2" s="3" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="T2" s="3" t="inlineStr">
+      <c r="U2" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="V2" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="V2" s="3" t="inlineStr">
-        <is>
-          <t>White</t>
-        </is>
-      </c>
       <c r="W2" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="X2" s="3" t="inlineStr">
         <is>
           <t>Tee time 8:30am. Fine autumn morning, light wind. Course in great condition. Happy with the round - hit it well off the tee, short game let me down on a few holes.</t>
         </is>
@@ -706,36 +713,38 @@
       <c r="F3" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
         <is>
           <t>Bogey</t>
         </is>
       </c>
-      <c r="H3" s="5" t="n">
+      <c r="I3" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="I3" s="5" t="n">
+      <c r="J3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="5" t="n">
+      <c r="K3" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="N3" s="5" t="inlineStr">
         <is>
           <t>Neutral</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr"/>
       <c r="O3" s="5" t="inlineStr"/>
       <c r="P3" s="5" t="inlineStr"/>
       <c r="Q3" s="5" t="inlineStr"/>
@@ -744,7 +753,8 @@
       <c r="T3" s="5" t="inlineStr"/>
       <c r="U3" s="5" t="inlineStr"/>
       <c r="V3" s="5" t="inlineStr"/>
-      <c r="W3" s="5" t="inlineStr">
+      <c r="W3" s="5" t="inlineStr"/>
+      <c r="X3" s="5" t="inlineStr">
         <is>
           <t>Good drive, approach came up short. Chip to 4m, two-putted.</t>
         </is>
@@ -773,36 +783,38 @@
       <c r="F4" s="5" t="n">
         <v>139</v>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="H4" s="5" t="n">
+      <c r="I4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="I4" s="5" t="n">
+      <c r="J4" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="5" t="n">
+      <c r="K4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>7 Iron</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr"/>
       <c r="O4" s="5" t="inlineStr"/>
       <c r="P4" s="5" t="inlineStr"/>
       <c r="Q4" s="5" t="inlineStr"/>
@@ -811,7 +823,8 @@
       <c r="T4" s="5" t="inlineStr"/>
       <c r="U4" s="5" t="inlineStr"/>
       <c r="V4" s="5" t="inlineStr"/>
-      <c r="W4" s="5" t="inlineStr">
+      <c r="W4" s="5" t="inlineStr"/>
+      <c r="X4" s="5" t="inlineStr">
         <is>
           <t>Solid tee shot to 3m, holed the putt. Exactly the plan.</t>
         </is>
@@ -840,36 +853,38 @@
       <c r="F5" s="5" t="n">
         <v>335</v>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
         <is>
           <t>Birdie</t>
         </is>
       </c>
-      <c r="H5" s="5" t="n">
+      <c r="I5" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="5" t="n">
+      <c r="J5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="J5" s="5" t="n">
+      <c r="K5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="L5" s="5" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr">
+      <c r="M5" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="M5" s="5" t="inlineStr">
+      <c r="N5" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
       <c r="O5" s="5" t="inlineStr"/>
       <c r="P5" s="5" t="inlineStr"/>
       <c r="Q5" s="5" t="inlineStr"/>
@@ -878,7 +893,8 @@
       <c r="T5" s="5" t="inlineStr"/>
       <c r="U5" s="5" t="inlineStr"/>
       <c r="V5" s="5" t="inlineStr"/>
-      <c r="W5" s="5" t="inlineStr">
+      <c r="W5" s="5" t="inlineStr"/>
+      <c r="X5" s="5" t="inlineStr">
         <is>
           <t>Big drive, wedge to 1.5m and holed it. Best hole of the day.</t>
         </is>
@@ -889,17 +905,14 @@
     <dataValidation sqref="C2:C9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Overall,Hole"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="L2:L9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Positive,Neutral,Negative"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Great,Good,Average,Poor"</formula1>
     </dataValidation>
     <dataValidation sqref="O2:O9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Great,Good,Average,Poor"</formula1>
@@ -919,7 +932,10 @@
     <dataValidation sqref="T2:T9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Great,Good,Average,Poor"</formula1>
     </dataValidation>
-    <dataValidation sqref="V2:V9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="U2:U9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Great,Good,Average,Poor"</formula1>
+    </dataValidation>
+    <dataValidation sqref="W2:W9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"White,Yellow,Red,Blue,Black"</formula1>
     </dataValidation>
   </dataValidations>
@@ -933,15 +949,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="6" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -957,20 +974,25 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Tee Colour</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Distance (m)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Stroke Index</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -985,16 +1007,21 @@
       <c r="B2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="F2" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1005,16 +1032,21 @@
       <c r="B3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="E3" s="3" t="n">
         <v>139</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="F3" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1025,16 +1057,21 @@
       <c r="B4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="E4" s="5" t="n">
         <v>335</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="F4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1045,16 +1082,21 @@
       <c r="B5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="C5" s="3" t="n">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="E5" s="3" t="n">
         <v>304</v>
       </c>
-      <c r="E5" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="F5" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1065,16 +1107,21 @@
       <c r="B6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="E6" s="5" t="n">
         <v>431</v>
       </c>
-      <c r="E6" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1085,16 +1132,21 @@
       <c r="B7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="C7" s="3" t="n">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="E7" s="3" t="n">
         <v>165</v>
       </c>
-      <c r="E7" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr"/>
+      <c r="F7" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1105,16 +1157,21 @@
       <c r="B8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="E8" s="5" t="n">
         <v>363</v>
       </c>
-      <c r="E8" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1125,16 +1182,21 @@
       <c r="B9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="C9" s="3" t="n">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="E9" s="3" t="n">
         <v>333</v>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr"/>
+      <c r="F9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1145,16 +1207,21 @@
       <c r="B10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="E10" s="5" t="n">
         <v>147</v>
       </c>
-      <c r="E10" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1165,16 +1232,21 @@
       <c r="B11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="C11" s="3" t="n">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="E11" s="3" t="n">
         <v>422</v>
       </c>
-      <c r="E11" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="F11" s="3" t="inlineStr"/>
+      <c r="F11" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="G11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1185,16 +1257,21 @@
       <c r="B12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="E12" s="5" t="n">
         <v>398</v>
       </c>
-      <c r="E12" s="5" t="n">
-        <v>18</v>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1205,16 +1282,21 @@
       <c r="B13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="C13" s="3" t="n">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="E13" s="3" t="n">
         <v>362</v>
       </c>
-      <c r="E13" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="3" t="inlineStr"/>
+      <c r="F13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1225,16 +1307,21 @@
       <c r="B14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="E14" s="5" t="n">
         <v>167</v>
       </c>
-      <c r="E14" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1245,16 +1332,21 @@
       <c r="B15" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="C15" s="3" t="n">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="E15" s="3" t="n">
         <v>285</v>
       </c>
-      <c r="E15" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F15" s="3" t="inlineStr"/>
+      <c r="F15" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1265,16 +1357,21 @@
       <c r="B16" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="E16" s="5" t="n">
         <v>299</v>
       </c>
-      <c r="E16" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1285,16 +1382,21 @@
       <c r="B17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="C17" s="3" t="n">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="E17" s="3" t="n">
         <v>238</v>
       </c>
-      <c r="E17" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F17" s="3" t="inlineStr"/>
+      <c r="F17" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1305,16 +1407,21 @@
       <c r="B18" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="E18" s="5" t="n">
         <v>143</v>
       </c>
-      <c r="E18" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1325,16 +1432,21 @@
       <c r="B19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="C19" s="3" t="n">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="E19" s="3" t="n">
         <v>357</v>
       </c>
-      <c r="E19" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
+      <c r="F19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1347,10 +1459,15 @@
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C20" s="6" t="n">
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="D20" s="6" t="n">
+      <c r="E20" s="6" t="n">
         <v>5188</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Guide tab, update hole notes, fix template/Drive separation
- Add Guide tab: score labels, sentiment guide, ball striking ratings
- Detailed hole-by-hole notes loaded for Pupuke 22-Feb-2026 round
- Hybrid rating corrected to Average
- create_workbook.py now saves to repo template only, never overwrites
  the live Drive file (prevents accidental data loss)
- README updated with Guide tab reference and sentiment/rating tables

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rounds" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,8 +42,25 @@
       <name val="Calibri"/>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +77,11 @@
         <fgColor rgb="00D9E8F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -72,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -82,6 +105,8 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1474,4 +1499,405 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>SCORE LABELS -- use these in the Score column for Hole rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Strokes vs Par</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Example (par 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Eagle</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>-2 or better</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>2 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Birdie</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>-1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>3 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Par</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>4 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Bogey</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>5 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Double Bogey</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>6 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Triple Bogey</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>7 strokes on a par 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>+4 or worse, or pick up</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>8+ strokes, or picked up</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>SENTIMENT -- how you felt the hole or round went</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Sentiment</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Your words might include...</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>great, best hole, happy, love it, exactly the plan, nice, solid, holed it</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>ok, sensible, got away with it, fine, average, recovered, not bad</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, awful, hack, lucky to escape, poor</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>BALL STRIKING RATINGS -- for Overall rows, one rating per club category</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="inlineStr">
+        <is>
+          <t>Your words might include...</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Great</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>good, solid, nice, decent, hit it well</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>duffed, hacked, bladed, hooked, sliced, below average, dire, terrible, sprayed</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>PICK UP -- did you finish the hole?</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Holed out -- counted every stroke</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Picked up / did not finish -- score is an estimate</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Notes should cover: tee time, weather, wind, course conditions, overall impressions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Score / Strokes = gross total for the round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Ball striking columns = how each club category felt across the whole round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Putts = total putts for the round (count all holes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Penalties = total penalty strokes for the round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Tee Colour = which tees played (affects par, distance, stroke index).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A24:C24"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add FIR, GIR, Course Rating, Slope, WHS Index columns
Rounds tab now 29 columns:
- FIR (col 12) and GIR (col 13) -- hole-level accuracy stats
- Course Rating (col 26), Slope (col 27), WHS Index (col 28) -- persisted
  on Overall rows so changes over time are captured

Courses tab now 9 columns:
- Course Rating and Slope added, populated on TOTAL row for each course/tee
- Pupuke White: Rating 68.2, Slope 119

Guide tab updated with FIR/GIR definitions and sentiment numeric scale
README and MEMORY.md updated throughout

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,11 +41,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -105,8 +100,8 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -472,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -486,19 +481,24 @@
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
     <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
-    <col width="11" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
-    <col width="60" customWidth="1" min="24" max="24"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="9" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
+    <col width="60" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -559,69 +559,96 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>FIR</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>GIR</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Tee Club</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Pick Up</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Sentiment</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Woods</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Hybrids</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Long Irons
 (5-7)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Short Irons
 (8-P)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Wedges
 (GW/SW/LW)</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Putter</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Playing
 Handicap</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Tee Colour</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Course
+Rating</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Slope</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>WHS
+Index</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -652,66 +679,75 @@
       </c>
       <c r="G2" s="3" t="n"/>
       <c r="H2" s="3" t="n">
-        <v>85</v>
+        <v>101</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>85</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="O2" s="3" t="inlineStr">
+        <v>101</v>
+      </c>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>Great</t>
+        </is>
+      </c>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="S2" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="T2" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="U2" s="3" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="V2" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="W2" s="3" t="inlineStr">
         <is>
           <t>Average</t>
         </is>
       </c>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="S2" s="3" t="inlineStr">
-        <is>
-          <t>Average</t>
-        </is>
-      </c>
-      <c r="T2" s="3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="U2" s="3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="V2" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="W2" s="3" t="inlineStr">
+      <c r="X2" s="3" t="n"/>
+      <c r="Y2" s="3" t="inlineStr">
         <is>
           <t>White</t>
         </is>
       </c>
-      <c r="X2" s="3" t="inlineStr">
-        <is>
-          <t>Tee time 8:30am. Fine autumn morning, light wind. Course in great condition. Happy with the round - hit it well off the tee, short game let me down on a few holes.</t>
+      <c r="Z2" s="3" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>119</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="AC2" s="3" t="inlineStr">
+        <is>
+          <t>Tee time 7:22am. Sample overall notes.</t>
         </is>
       </c>
     </row>
@@ -730,220 +766,91 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E3" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>300</v>
+        <v>304</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Bogey</t>
+          <t>Par</t>
         </is>
       </c>
       <c r="I3" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="K3" s="5" t="n">
-        <v>0</v>
-      </c>
+      <c r="K3" s="5" t="n"/>
       <c r="L3" s="5" t="inlineStr">
         <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="M3" s="5" t="inlineStr">
+      <c r="O3" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>Neutral</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr"/>
-      <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr"/>
-      <c r="R3" s="5" t="inlineStr"/>
-      <c r="S3" s="5" t="inlineStr"/>
-      <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="5" t="inlineStr"/>
-      <c r="V3" s="5" t="inlineStr"/>
-      <c r="W3" s="5" t="inlineStr"/>
-      <c r="X3" s="5" t="inlineStr">
-        <is>
-          <t>Good drive, approach came up short. Chip to 4m, two-putted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="4" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Pupuke</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Hole</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>139</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>15</v>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Par</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>7 Iron</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="P3" s="5" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr"/>
-      <c r="R4" s="5" t="inlineStr"/>
-      <c r="S4" s="5" t="inlineStr"/>
-      <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="5" t="inlineStr"/>
-      <c r="V4" s="5" t="inlineStr"/>
-      <c r="W4" s="5" t="inlineStr"/>
-      <c r="X4" s="5" t="inlineStr">
-        <is>
-          <t>Solid tee shot to 3m, holed the putt. Exactly the plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
-        <v>46075</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Pupuke</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Hole</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>335</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Birdie</t>
-        </is>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>Driver</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr"/>
-      <c r="R5" s="5" t="inlineStr"/>
-      <c r="S5" s="5" t="inlineStr"/>
-      <c r="T5" s="5" t="inlineStr"/>
-      <c r="U5" s="5" t="inlineStr"/>
-      <c r="V5" s="5" t="inlineStr"/>
-      <c r="W5" s="5" t="inlineStr"/>
-      <c r="X5" s="5" t="inlineStr">
-        <is>
-          <t>Big drive, wedge to 1.5m and holed it. Best hole of the day.</t>
+      <c r="Q3" s="5" t="n"/>
+      <c r="R3" s="5" t="n"/>
+      <c r="S3" s="5" t="n"/>
+      <c r="T3" s="5" t="n"/>
+      <c r="U3" s="5" t="n"/>
+      <c r="V3" s="5" t="n"/>
+      <c r="W3" s="5" t="n"/>
+      <c r="X3" s="5" t="n"/>
+      <c r="Y3" s="5" t="n"/>
+      <c r="Z3" s="5" t="n"/>
+      <c r="AA3" s="5" t="n"/>
+      <c r="AB3" s="5" t="n"/>
+      <c r="AC3" s="5" t="inlineStr">
+        <is>
+          <t>Good drive, good PW onto green, two putt.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
+  <dataValidations count="14">
     <dataValidation sqref="C2:C9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Overall,Hole"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Other"</formula1>
     </dataValidation>
+    <dataValidation sqref="L2:L9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
     <dataValidation sqref="M2:M9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Positive,Neutral,Negative"</formula1>
-    </dataValidation>
     <dataValidation sqref="O2:O9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Great,Good,Average,Poor"</formula1>
+      <formula1>"Y,N"</formula1>
     </dataValidation>
     <dataValidation sqref="P2:P9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Great,Good,Average,Poor"</formula1>
+      <formula1>"Positive,Neutral,Negative"</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Great,Good,Average,Poor"</formula1>
@@ -960,7 +867,13 @@
     <dataValidation sqref="U2:U9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Great,Good,Average,Poor"</formula1>
     </dataValidation>
+    <dataValidation sqref="V2:V9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Great,Good,Average,Poor"</formula1>
+    </dataValidation>
     <dataValidation sqref="W2:W9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Great,Good,Average,Poor"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Y2:Y9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"White,Yellow,Red,Blue,Black"</formula1>
     </dataValidation>
   </dataValidations>
@@ -974,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -983,7 +896,9 @@
     <col width="6" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1019,6 +934,16 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Course Rating</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Slope</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
@@ -1046,7 +971,9 @@
       <c r="F2" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1071,7 +998,9 @@
       <c r="F3" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G3" s="3" t="inlineStr"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -1096,7 +1025,9 @@
       <c r="F4" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -1121,7 +1052,9 @@
       <c r="F5" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="G5" s="3" t="inlineStr"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -1146,7 +1079,9 @@
       <c r="F6" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="5" t="n"/>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -1171,7 +1106,9 @@
       <c r="F7" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="G7" s="3" t="inlineStr"/>
+      <c r="G7" s="3" t="n"/>
+      <c r="H7" s="3" t="n"/>
+      <c r="I7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1196,7 +1133,9 @@
       <c r="F8" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -1221,7 +1160,9 @@
       <c r="F9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="3" t="inlineStr"/>
+      <c r="G9" s="3" t="n"/>
+      <c r="H9" s="3" t="n"/>
+      <c r="I9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1246,7 +1187,9 @@
       <c r="F10" s="5" t="n">
         <v>17</v>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="H10" s="5" t="n"/>
+      <c r="I10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1271,7 +1214,9 @@
       <c r="F11" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="G11" s="3" t="inlineStr"/>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1296,7 +1241,9 @@
       <c r="F12" s="5" t="n">
         <v>16</v>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="H12" s="5" t="n"/>
+      <c r="I12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -1321,7 +1268,9 @@
       <c r="F13" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="3" t="inlineStr"/>
+      <c r="G13" s="3" t="n"/>
+      <c r="H13" s="3" t="n"/>
+      <c r="I13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1346,7 +1295,9 @@
       <c r="F14" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="H14" s="5" t="n"/>
+      <c r="I14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1371,7 +1322,9 @@
       <c r="F15" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="G15" s="3" t="inlineStr"/>
+      <c r="G15" s="3" t="n"/>
+      <c r="H15" s="3" t="n"/>
+      <c r="I15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1396,7 +1349,9 @@
       <c r="F16" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -1421,7 +1376,9 @@
       <c r="F17" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="G17" s="3" t="inlineStr"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1446,7 +1403,9 @@
       <c r="F18" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
@@ -1471,7 +1430,9 @@
       <c r="F19" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="3" t="inlineStr"/>
+      <c r="G19" s="3" t="n"/>
+      <c r="H19" s="3" t="n"/>
+      <c r="I19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1495,6 +1456,14 @@
       <c r="E20" s="6" t="n">
         <v>5188</v>
       </c>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>119</v>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1507,18 +1476,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C35"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>SCORE LABELS -- use these in the Score column for Hole rows</t>
+          <t>SCORE LABELS -- Score column on Hole rows</t>
         </is>
       </c>
     </row>
@@ -1654,26 +1623,26 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>8+ strokes, or picked up</t>
+          <t>8+ strokes or picked up</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>SENTIMENT -- how you felt the hole or round went</t>
+          <t>FIR -- Fairway in Regulation (par 4s and 5s only, leave blank on par 3s and Overall)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Sentiment</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Your words might include...</t>
+          <t>Meaning</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr"/>
@@ -1681,12 +1650,12 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>great, best hole, happy, love it, exactly the plan, nice, solid, holed it</t>
+          <t>Tee shot landed on the fairway</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr"/>
@@ -1694,12 +1663,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>ok, sensible, got away with it, fine, average, recovered, not bad</t>
+          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -1707,12 +1676,12 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, awful, hack, lucky to escape, poor</t>
+          <t>Par 3 tee shots and Overall rows</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr"/>
@@ -1720,104 +1689,116 @@
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>BALL STRIKING RATINGS -- for Overall rows, one rating per club category</t>
+          <t>GIR -- Green in Regulation (all hole rows, leave blank on Overall)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Rating</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Your words might include...</t>
-        </is>
-      </c>
-      <c r="C18" s="8" t="inlineStr"/>
+          <t>Meaning</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Regulation shots to green</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Great</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr"/>
+          <t>Ball on putting surface within regulation</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>N</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>good, solid, nice, decent, hit it well</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr"/>
+          <t>Missed the green in regulation</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Chipping / pitching in = N</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>(blank)</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+          <t>Pick up holes and Overall rows</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr"/>
     </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Poor</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>duffed, hacked, bladed, hooked, sliced, below average, dire, terrible, sprayed</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
-        <is>
-          <t>PICK UP -- did you finish the hole?</t>
-        </is>
-      </c>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>SENTIMENT -- how you felt the hole or round went</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Your words might include...</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Meaning</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr"/>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Neutral</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Holed out -- counted every stroke</t>
+          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
@@ -1825,12 +1806,12 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Picked up / did not finish -- score is an estimate</t>
+          <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, hack, awful, poor</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr"/>
@@ -1838,65 +1819,212 @@
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
+          <t>BALL STRIKING RATINGS -- Overall rows, one rating per club category</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Notes should cover: tee time, weather, wind, course conditions, overall impressions.</t>
+      <c r="A30" s="8" t="inlineStr">
+        <is>
+          <t>Rating</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>Your words might include...</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>Numeric (PBI)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Score / Strokes = gross total for the round.</t>
+          <t>Great</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Ball striking columns = how each club category felt across the whole round.</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>good, solid, nice, decent, hit it well</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Putts = total putts for the round (count all holes).</t>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Penalties = total penalty strokes for the round.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>Tee Colour = which tees played (affects par, distance, stroke index).</t>
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Poor</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>duffed, hacked, bladed, hooked, sliced, below average, dire</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>SENTIMENT NUMERIC SCALE (for Power BI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Numeric</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>Score / Strokes = gross total for the round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>Ball striking = how each club category felt across the whole round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Putts / Penalties = total for the round.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A33:C33"/>
+  <mergeCells count="13">
+    <mergeCell ref="A42:C42"/>
+    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A46:C46"/>
     <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A34:C34"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A43:C43"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add How To tab, schema change workflow to README
- How To tab in workbook mirrors README operational notes:
  file locations, round entry steps, schema change procedure,
  adding courses, Power BI notes
- README Workflow section updated with schema change gotcha:
  must copy template to Drive before reloading data or columns misalign
- Both updated together so they stay in sync via source control

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rounds" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Courses" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -53,6 +54,11 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="5">
@@ -90,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,6 +108,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2028,4 +2042,411 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>FILE LOCATIONS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="9" t="inlineStr"/>
+      <c r="B2" s="9" t="inlineStr">
+        <is>
+          <t>Live data file (edit here)</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>G:\My Drive\Project_Outputs\Golf Round Recap\Golf Round Recap.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="11" t="inlineStr"/>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>Base template (source control)</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>C:\Users\craig.f\Home_Projects\Golf Round Recap\Golf Round Recap.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="9" t="inlineStr"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>GitHub repo</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>https://github.com/C-Fowler-Tech/golf-round-recap</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>ENTERING A NEW ROUND</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Open live file</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>G:\My Drive\Project_Outputs\Golf Round Recap\Golf Round Recap.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>Add Overall row</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>Note Type = Overall, Hole = 0. Fill date, course, tee colour, gross score, playing handicap, course rating, slope, WHS index, ball striking ratings, notes (tee time, weather, conditions, overall impressions).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Add Hole rows</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>One row per hole. Note Type = Hole. Fill par, distance, stroke index from the Courses tab. Fill FIR (par 4/5 only), GIR, score, strokes, putts, penalties, tee club, pick up, sentiment, notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>Save</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>OneDrive AutoSave handles sync. No manual save needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Commit to git (optional)</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>After a data entry session, commit the Drive file for backup history:
+git add . &amp;&amp; git commit -m 'Add round: Pupuke DD-Mon-YYYY' &amp;&amp; git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>CHANGING THE SCHEMA (adding/removing columns)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="28" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="inlineStr">
+        <is>
+          <t>Update create_workbook.py</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>Add the new column to ROUND_HEADERS, ROUND_COL_WIDTHS, sample rows, and data validations. Update Guide tab content if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Run create_workbook.py</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Saves new template to repo only -- does NOT touch the Drive file.
+cd 'C:\Users\craig.f\Home_Projects\Golf Round Recap'
+python create_workbook.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="inlineStr">
+        <is>
+          <t>Copy template to Drive</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>MUST do this before reloading data, otherwise data lands in wrong columns.
+python -c "import shutil; shutil.copy2('Golf Round Recap.xlsx', r'G:\My Drive\Project_Outputs\Golf Round Recap\Golf Round Recap.xlsx')\"</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="28" customHeight="1">
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Reload data</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Run any data loading scripts (e.g. load_round_YYYYMMDD.py) after the template has been copied. Data will now align to the new schema.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>Update README.md</t>
+        </is>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>Keep the column guide in README.md in sync with the workbook. Both live in source control -- update together in the same commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="28" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Commit everything</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>git add . &amp;&amp; git commit -m 'Schema: describe change' &amp;&amp; git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>ADDING A NEW COURSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="28" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Open Courses tab</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t>Add 18 rows (one per hole) for the new course and tee colour.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Fill columns</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Course name must match EXACTLY what you will type in the Rounds tab. Fill Hole, Tee Colour, Par, Distance (m), Stroke Index. On the TOTAL row, fill Course Rating and Slope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Update create_workbook.py</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t>Add the course data to the script so it is included in future template resets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>POWER BI</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="A27" s="11" t="inlineStr"/>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Data source</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Connect to G:\My Drive\Project_Outputs\Golf Round Recap\Golf Round Recap.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="A28" s="9" t="inlineStr"/>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>Rounds grain</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t>Filter Note Type = 'Overall' for round-level measures. Filter Note Type = 'Hole' for hole-level measures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="28" customHeight="1">
+      <c r="A29" s="11" t="inlineStr"/>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>Sentiment (numeric)</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Positive = 5, Neutral = 3, Negative = 1  (calculated column in PBI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="28" customHeight="1">
+      <c r="A30" s="9" t="inlineStr"/>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>Ball striking (numeric)</t>
+        </is>
+      </c>
+      <c r="C30" s="10" t="inlineStr">
+        <is>
+          <t>Great = 4, Good = 3, Average = 2, Poor = 1  (calculated column in PBI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="28" customHeight="1">
+      <c r="A31" s="11" t="inlineStr"/>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Handicap differential</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Formula: (Score - Course Rating) x 113 / Slope</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A26:C26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add Pick Up to Score dropdown
Clearer than Other for holes where you didn't finish.
Updated dropdown, Guide tab, score_label function, and README.
Holes 12 and 13 now correctly show Pick Up in score column.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -852,7 +852,7 @@
       <formula1>"Overall,Hole"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Other"</formula1>
+      <formula1>"Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Pick Up,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -1490,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C48"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1627,62 +1627,66 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>Pick Up</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Did not finish hole</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>Use with Pick Up column = Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>+4 or worse, or pick up</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>8+ strokes or picked up</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>+4 or worse</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>8+ strokes, no pick up</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>FIR -- Fairway in Regulation (par 4s and 5s only, leave blank on par 3s and Overall)</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Tee shot landed on the fairway</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr"/>
+      <c r="C13" s="8" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+          <t>Tee shot landed on the fairway</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -1690,129 +1694,129 @@
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Par 3 tee shots and Overall rows</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>GIR -- Green in Regulation (all hole rows, leave blank on Overall)</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>Regulation shots to green</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Ball on putting surface within regulation</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Missed the green in regulation</t>
+          <t>Ball on putting surface within regulation</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Chipping / pitching in = N</t>
+          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Missed the green in regulation</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Chipping / pitching in = N</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Pick up holes and Overall rows</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT -- how you felt the hole or round went</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B25" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr"/>
+      <c r="C25" s="8" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
@@ -1820,225 +1824,238 @@
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, hack, awful, poor</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr"/>
-    </row>
-    <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="7" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>BALL STRIKING RATINGS -- Overall rows, one rating per club category</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C31" s="8" t="inlineStr">
         <is>
           <t>Numeric (PBI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Great</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Great</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>good, solid, nice, decent, hit it well</t>
+          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+          <t>good, solid, nice, decent, hit it well</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
           <t>Poor</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>duffed, hacked, bladed, hooked, sliced, below average, dire</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="20" customHeight="1">
-      <c r="A36" s="7" t="inlineStr">
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT NUMERIC SCALE (for Power BI)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t>Numeric</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B38" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C38" s="3" t="inlineStr"/>
+      <c r="C38" s="8" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B39" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B40" s="3" t="n">
+      <c r="B41" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C40" s="3" t="inlineStr"/>
-    </row>
-    <row r="42" ht="20" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Score / Strokes = gross total for the round.</t>
+          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
+          <t>Score / Strokes = gross total for the round.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
+          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Ball striking = how each club category felt across the whole round.</t>
+          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
+          <t>Ball striking = how each club category felt across the whole round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
           <t>Putts / Penalties = total for the round.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A42:C42"/>
-    <mergeCell ref="A36:C36"/>
-    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A48:C48"/>
     <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A24:C24"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Hole in One to Score dropdown
Because Other was a deeply underwhelming way to record it.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -852,7 +852,7 @@
       <formula1>"Overall,Hole"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Pick Up,Other"</formula1>
+      <formula1>"Hole in One,Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Pick Up,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -1490,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1525,181 +1525,185 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Eagle</t>
+          <t>Hole in One</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>-2 or better</t>
+          <t>-2 or better (par 3)</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>2 strokes on a par 4</t>
+          <t>1 stroke on a par 3 -- the dream</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Birdie</t>
+          <t>Eagle</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-2 or better</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>3 strokes on a par 4</t>
+          <t>2 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Par</t>
+          <t>Birdie</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>4 strokes on a par 4</t>
+          <t>3 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Bogey</t>
+          <t>Par</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>5 strokes on a par 4</t>
+          <t>4 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Double Bogey</t>
+          <t>Bogey</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>6 strokes on a par 4</t>
+          <t>5 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Triple Bogey</t>
+          <t>Double Bogey</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>7 strokes on a par 4</t>
+          <t>6 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Pick Up</t>
+          <t>Triple Bogey</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Did not finish hole</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Use with Pick Up column = Y</t>
+          <t>7 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>Pick Up</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Did not finish hole</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Use with Pick Up column = Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>+4 or worse</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>8+ strokes, no pick up</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>FIR -- Fairway in Regulation (par 4s and 5s only, leave blank on par 3s and Overall)</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Tee shot landed on the fairway</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr"/>
+      <c r="C14" s="8" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+          <t>Tee shot landed on the fairway</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr"/>
@@ -1707,129 +1711,129 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B17" s="5" t="inlineStr">
         <is>
           <t>Par 3 tee shots and Overall rows</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>GIR -- Green in Regulation (all hole rows, leave blank on Overall)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>Regulation shots to green</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Ball on putting surface within regulation</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Missed the green in regulation</t>
+          <t>Ball on putting surface within regulation</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Chipping / pitching in = N</t>
+          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Missed the green in regulation</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Chipping / pitching in = N</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Pick up holes and Overall rows</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT -- how you felt the hole or round went</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B26" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr"/>
+      <c r="C26" s="8" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr"/>
@@ -1837,225 +1841,238 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, hack, awful, poor</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>BALL STRIKING RATINGS -- Overall rows, one rating per club category</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="8" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B32" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Numeric (PBI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>Great</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>4</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Great</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>good, solid, nice, decent, hit it well</t>
+          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+          <t>good, solid, nice, decent, hit it well</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
           <t>Poor</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>duffed, hacked, bladed, hooked, sliced, below average, dire</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="20" customHeight="1">
-      <c r="A37" s="7" t="inlineStr">
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT NUMERIC SCALE (for Power BI)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="8" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t>Numeric</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C39" s="5" t="inlineStr"/>
+      <c r="C39" s="8" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C40" s="3" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" s="5" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B41" s="5" t="n">
+      <c r="B42" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C41" s="5" t="inlineStr"/>
-    </row>
-    <row r="43" ht="20" customHeight="1">
-      <c r="A43" s="7" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
-          <t>Score / Strokes = gross total for the round.</t>
+          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
+          <t>Score / Strokes = gross total for the round.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
+          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Ball striking = how each club category felt across the whole round.</t>
+          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
+          <t>Ball striking = how each club category felt across the whole round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
           <t>Putts / Penalties = total for the round.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A44:C44"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A37:C37"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A49:C49"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A50:C50"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A43:C43"/>
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A38:C38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add Albatross to Score dropdown (not Double Eagle, we're not savages)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Golf Round Recap.xlsx
+++ b/Golf Round Recap.xlsx
@@ -852,7 +852,7 @@
       <formula1>"Overall,Hole"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Hole in One,Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Pick Up,Other"</formula1>
+      <formula1>"Hole in One,Albatross,Eagle,Birdie,Par,Bogey,Double Bogey,Triple Bogey,Pick Up,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L9999" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -1490,7 +1490,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C50"/>
+  <dimension ref="A1:C51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1542,181 +1542,185 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Eagle</t>
+          <t>Albatross</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>-2 or better</t>
+          <t>-3</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2 strokes on a par 4</t>
+          <t>2 strokes on a par 5</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Birdie</t>
+          <t>Eagle</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>-1</t>
+          <t>-2</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>3 strokes on a par 4</t>
+          <t>2 strokes on a par 4, 3 on a par 5</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Par</t>
+          <t>Birdie</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>-1</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>4 strokes on a par 4</t>
+          <t>3 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Bogey</t>
+          <t>Par</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>+1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>5 strokes on a par 4</t>
+          <t>4 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Double Bogey</t>
+          <t>Bogey</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>+2</t>
+          <t>+1</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>6 strokes on a par 4</t>
+          <t>5 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Triple Bogey</t>
+          <t>Double Bogey</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>+3</t>
+          <t>+2</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>7 strokes on a par 4</t>
+          <t>6 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Pick Up</t>
+          <t>Triple Bogey</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Did not finish hole</t>
+          <t>+3</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Use with Pick Up column = Y</t>
+          <t>7 strokes on a par 4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Pick Up</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Did not finish hole</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Use with Pick Up column = Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>Other</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>+4 or worse</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>8+ strokes, no pick up</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>FIR -- Fairway in Regulation (par 4s and 5s only, leave blank on par 3s and Overall)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B15" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Tee shot landed on the fairway</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr"/>
+      <c r="C15" s="8" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+          <t>Tee shot landed on the fairway</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
@@ -1724,129 +1728,129 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Tee shot missed fairway (rough, bunker, OB, etc.)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr">
         <is>
           <t>Par 3 tee shots and Overall rows</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr"/>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>GIR -- Green in Regulation (all hole rows, leave blank on Overall)</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B21" s="8" t="inlineStr">
         <is>
           <t>Meaning</t>
         </is>
       </c>
-      <c r="C20" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Regulation shots to green</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>Ball on putting surface within regulation</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Missed the green in regulation</t>
+          <t>Ball on putting surface within regulation</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Chipping / pitching in = N</t>
+          <t>Par 3 = tee shot | Par 4 = within 2 | Par 5 = within 3</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Missed the green in regulation</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Chipping / pitching in = N</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
           <t>(blank)</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Pick up holes and Overall rows</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT -- how you felt the hole or round went</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr"/>
+      <c r="C27" s="8" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+          <t>great, best hole, happy, exactly the plan, nice, solid, holed it, love it</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
@@ -1854,225 +1858,238 @@
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>ok, sensible, got away with it, fine, recovered, not bad, average</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>disappointed, disaster, terrible, nightmare, duffed, dire, struggled, hack, awful, poor</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr"/>
-    </row>
-    <row r="31" ht="20" customHeight="1">
-      <c r="A31" s="7" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>BALL STRIKING RATINGS -- Overall rows, one rating per club category</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>Your words might include...</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="C33" s="8" t="inlineStr">
         <is>
           <t>Numeric (PBI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Great</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Great</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>good, solid, nice, decent, hit it well</t>
+          <t>monster, perfect, very good, flushed it, exactly where I wanted</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Average</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+          <t>good, solid, nice, decent, hit it well</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
+          <t>Average</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>ok, bit fadey, slight fade/slice, average, could be better</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
           <t>Poor</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>duffed, hacked, bladed, hooked, sliced, below average, dire</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="20" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>SENTIMENT NUMERIC SCALE (for Power BI)</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="8" t="inlineStr">
         <is>
           <t>Text</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B40" s="8" t="inlineStr">
         <is>
           <t>Numeric</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C40" s="3" t="inlineStr"/>
+      <c r="C40" s="8" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Neutral</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="B41" s="5" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="B42" s="3" t="n">
+      <c r="B43" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
-    </row>
-    <row r="44" ht="20" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>OVERALL ROW TIPS -- one per round, Hole = 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
         <is>
-          <t>Score / Strokes = gross total for the round.</t>
+          <t>Notes: tee time, weather, wind, course conditions, overall impressions.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
+          <t>Score / Strokes = gross total for the round.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
+          <t>FIR / GIR = leave blank on Overall rows (fill totals in notes if wanted).</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Ball striking = how each club category felt across the whole round.</t>
+          <t>Course Rating, Slope, WHS Index = persist here so changes over time are captured.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
+          <t>Ball striking = how each club category felt across the whole round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
           <t>Putts / Penalties = total for the round.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A49:C49"/>
     <mergeCell ref="A47:C47"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A45:C45"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A46:C46"/>
-    <mergeCell ref="A49:C49"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="A50:C50"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A39:C39"/>
+    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A51:C51"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>